<commit_message>
sync: actuary · 2026-07-14 08:35:35
</commit_message>
<xml_diff>
--- a/fase_1/lista_cruda/tabulador.xlsx
+++ b/fase_1/lista_cruda/tabulador.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
@@ -47,6 +47,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -68,11 +69,13 @@
       <color rgb="FFFFFFFF"/>
       <name val="Inter"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Inter"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -128,15 +131,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>